<commit_message>
NRT fix Excel suite_test_pec: allinea nomi funzione a file reali (conservazione_02, accessi_01, fatture_01)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/suite_test_pec.xlsx
+++ b/suite_test_pec.xlsx
@@ -355,7 +355,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -391,11 +391,44 @@
         <color rgb="00BFBFBF"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="170">
+  <cellXfs count="171">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -902,6 +935,7 @@
     <xf numFmtId="0" fontId="35" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1481,6 +1515,7 @@
           <t>TOTALE CASI DI TEST</t>
         </is>
       </c>
+      <c r="B14" s="170" t="n"/>
       <c r="C14" s="22" t="n">
         <v>65</v>
       </c>
@@ -1559,7 +1594,7 @@
       <c r="B3" s="157" t="inlineStr">
         <is>
           <t>test_fatture_01.py
-test_visualizza_fattura_importata</t>
+test_import_fattura_ricevute</t>
         </is>
       </c>
       <c r="C3" s="158" t="inlineStr">
@@ -1696,7 +1731,7 @@
       <c r="B3" s="165" t="inlineStr">
         <is>
           <t>test_accessi_01.py
-test_panoramica_accessi</t>
+test_panoramica_accessi_altri_account</t>
         </is>
       </c>
       <c r="C3" s="166" t="inlineStr">
@@ -4389,7 +4424,7 @@
       </c>
       <c r="D62" s="34" t="inlineStr">
         <is>
-          <t>test_conservazione_da_waffle</t>
+          <t>test_conservazione_waffle_menu</t>
         </is>
       </c>
       <c r="E62" s="35" t="inlineStr">
@@ -4432,7 +4467,7 @@
       </c>
       <c r="D63" s="82" t="inlineStr">
         <is>
-          <t>test_visualizza_fattura_importata</t>
+          <t>test_import_fattura_ricevute</t>
         </is>
       </c>
       <c r="E63" s="83" t="inlineStr">
@@ -4521,7 +4556,7 @@
       </c>
       <c r="D65" s="89" t="inlineStr">
         <is>
-          <t>test_panoramica_accessi</t>
+          <t>test_panoramica_accessi_altri_account</t>
         </is>
       </c>
       <c r="E65" s="90" t="inlineStr">
@@ -7126,7 +7161,7 @@
       <c r="B4" s="102" t="inlineStr">
         <is>
           <t>test_conservazione_02.py
-test_conservazione_da_waffle</t>
+test_conservazione_waffle_menu</t>
         </is>
       </c>
       <c r="C4" s="103" t="inlineStr">

</xml_diff>

<commit_message>
docs(excel-suite): sposta 'Scattare screenshot' prima degli assert nei passi di tutti i test (PEL/PEC/Mobile)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/suite_test_pec.xlsx
+++ b/suite_test_pec.xlsx
@@ -1579,8 +1579,8 @@
 8. Attendere il file input (#hidden_input) e impostare il file EML di test.
 9. Attendere il messaggio di conferma importazione.
 10. Navigare a 'Fatture ricevute'.
-11. Verificare che sia presente almeno un messaggio con riferimento a SDI o FatturaPA.
-12. Scattare screenshot.</t>
+11. Scattare screenshot.
+12. Verificare che sia presente almeno un messaggio con riferimento a SDI o FatturaPA (assert).</t>
         </is>
       </c>
       <c r="E3" s="85" t="inlineStr">
@@ -1614,8 +1614,8 @@
 5. Navigare direttamente a /new/settings/read-invoices.
 6. Verificare che la pagina si carichi (stato domcontentloaded).
 7. Verificare la presenza dell'h1 o testo 'Leggi fatture'.
-8. Verificare la presenza di contenuto informativo (cassetto fiscale, AdE, ecc.).
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la presenza di contenuto informativo (cassetto fiscale, AdE, ecc., assert).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">
@@ -1715,8 +1715,8 @@
 7. Verificare la presenza di almeno 2 pulsanti 'Gestisci'.
 8. Navigare alla sotto-sezione Multiutente PEC e verificare il contenuto.
 9. Tornare alla panoramica e navigare a Supervisore360.
-10. Verificare il contenuto della sezione Supervisore360.
-11. Scattare screenshot.</t>
+10. Scattare screenshot.
+11. Verificare il contenuto della sezione Supervisore360 (assert).</t>
         </is>
       </c>
       <c r="E3" s="92" t="inlineStr">
@@ -1751,8 +1751,8 @@
 6. Cercare e cliccare il pulsante 'Aggiungi' (multi-fallback selectors).
 7. Skip se il pulsante non e' trovato (pytest.skip).
 8. Verificare che il form o dialog si sia aperto con campi input.
-9. Chiudere il form senza inviare (tasto Annulla o Escape).
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Chiudere il form senza inviare (tasto Annulla o Escape).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">
@@ -1788,8 +1788,8 @@
 7. Cercare e cliccare il pulsante 'Aggiungi' o 'Nuova delega' (multi-fallback selectors).
 8. Skip se il pulsante non e' trovato (pytest.skip).
 9. Verificare che il form o dialog si sia aperto con campi email/input.
-10. Chiudere il form senza inviare (tasto Annulla o Escape).
-11. Scattare screenshot.</t>
+10. Scattare screenshot.
+11. Chiudere il form senza inviare (tasto Annulla o Escape).</t>
         </is>
       </c>
       <c r="E5" s="92" t="inlineStr">
@@ -1900,8 +1900,8 @@
 3. Cliccare il pulsante dell'account (username).
 4. Cliccare il pulsante 'Esci' dal menu dropdown.
 5. Attendere il reindirizzamento alla pagina di login.
-6. Verificare che il campo username sia visibile.
-7. Scattare screenshot della pagina di login.</t>
+6. Scattare screenshot della pagina di login.
+7. Verificare che il campo username sia visibile (assert).</t>
         </is>
       </c>
       <c r="G3" s="31" t="inlineStr">
@@ -1943,8 +1943,8 @@
 5. Cliccare il pulsante Login.
 6. Attendere 2 secondi.
 7. Verificare che l'URL non contenga 'INBOX'.
-8. Verificare la visibilità del messaggio di errore.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la visibilità del messaggio di errore (assert).</t>
         </is>
       </c>
       <c r="G4" s="37" t="inlineStr">
@@ -1987,8 +1987,8 @@
 6. Inviare il messaggio.
 7. Attendere la ricezione nella cartella In arrivo.
 8. Aprire il messaggio ricevuto.
-9. Verificare la presenza dell'allegato nel messaggio.
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Verificare la presenza dell'allegato nel messaggio (assert).</t>
         </is>
       </c>
       <c r="G5" s="43" t="inlineStr">
@@ -2030,8 +2030,8 @@
 5. Cliccare il pulsante 'Inoltra'.
 6. Inserire il destinatario dell'inoltro.
 7. Inviare il messaggio inoltrato.
-8. Verificare la comparsa del toast di conferma.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la comparsa del toast di conferma (assert).</t>
         </is>
       </c>
       <c r="G6" s="37" t="inlineStr">
@@ -2113,8 +2113,8 @@
 3. Selezionare il file da importare.
 4. Avviare il processo di importazione.
 5. Attendere il completamento dell'importazione.
-6. Verificare il messaggio di conferma.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare il messaggio di conferma (assert).</t>
         </is>
       </c>
       <c r="G8" s="37" t="inlineStr">
@@ -2155,8 +2155,8 @@
 4. Rinominare la cartella con un nuovo nome.
 5. Verificare il toast di conferma della modifica.
 6. Eliminare la cartella.
-7. Verificare il toast di conferma dell'eliminazione.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare il toast di conferma dell'eliminazione (assert).</t>
         </is>
       </c>
       <c r="G9" s="43" t="inlineStr">
@@ -2197,8 +2197,8 @@
 4. Selezionare il/i messaggio/i da ripristinare.
 5. Cliccare 'Ripristina' o 'Sposta in In arrivo'.
 6. Verificare che i messaggi non siano più nel cestino.
-7. Navigare in In arrivo e verificare la presenza dei messaggi.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Navigare in In arrivo e verificare la presenza dei messaggi (assert).</t>
         </is>
       </c>
       <c r="G10" s="37" t="inlineStr">
@@ -2238,8 +2238,8 @@
 3. Aggiungere il messaggio ai preferiti (stella).
 4. Verificare che il messaggio compaia nella cartella Preferiti/Speciali.
 5. Selezionare un messaggio e cliccare 'Pinna messaggio'.
-6. Verificare la presenza del messaggio pinnato.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare la presenza del messaggio pinnato (assert).</t>
         </is>
       </c>
       <c r="G11" s="43" t="inlineStr">
@@ -2280,8 +2280,8 @@
 4. Tornare in In arrivo e selezionare un messaggio.
 5. Applicare l'etichetta appena creata al messaggio.
 6. Verificare che l'etichetta sia visibile sul messaggio.
-7. Eliminare l'etichetta.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Eliminare l'etichetta (cleanup).</t>
         </is>
       </c>
       <c r="G12" s="37" t="inlineStr">
@@ -2321,8 +2321,8 @@
 3. Cliccare 'Segna come letto'.
 4. Verificare che il messaggio non sia più in grassetto (letto).
 5. Cliccare 'Segna come da leggere' sullo stesso messaggio.
-6. Verificare che il messaggio torni in grassetto (non letto).
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il messaggio torni in grassetto (non letto, assert).</t>
         </is>
       </c>
       <c r="G13" s="43" t="inlineStr">
@@ -2364,8 +2364,8 @@
 5. Inviare il messaggio.
 6. Attendere la ricezione in In arrivo.
 7. Aprire il messaggio ricevuto.
-8. Verificare la presenza dell'indicatore di alta priorità.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la presenza dell'indicatore di alta priorità (assert).</t>
         </is>
       </c>
       <c r="G14" s="37" t="inlineStr">
@@ -2447,8 +2447,8 @@
 3. Inserire l'indirizzo del destinatario.
 4. Inserire oggetto e corpo del messaggio.
 5. Cliccare 'Invia'.
-6. Verificare la comparsa del toast di conferma invio.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare la comparsa del toast di conferma invio (assert).</t>
         </is>
       </c>
       <c r="G16" s="37" t="inlineStr">
@@ -2531,8 +2531,8 @@
 3. Attendere la ricezione del messaggio.
 4. Selezionare il messaggio e cliccare 'Elimina'.
 5. Navigare nella cartella Cestino.
-6. Verificare che il messaggio eliminato sia presente nel cestino.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il messaggio eliminato sia presente nel cestino (assert).</t>
         </is>
       </c>
       <c r="G18" s="37" t="inlineStr">
@@ -2574,8 +2574,8 @@
 5. Selezionare il messaggio e cliccare 'Sposta in...'.
 6. Selezionare la cartella di destinazione.
 7. Verificare che il messaggio non sia più in In arrivo.
-8. Navigare nella cartella di destinazione e verificare la presenza del messaggio.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Navigare nella cartella di destinazione e verificare la presenza del messaggio (assert).</t>
         </is>
       </c>
       <c r="G19" s="43" t="inlineStr">
@@ -2616,8 +2616,8 @@
 4. Selezionare 'Copia in...' dal menu azioni.
 5. Selezionare la cartella di destinazione.
 6. Verificare che il messaggio originale sia ancora in In arrivo.
-7. Navigare nella cartella di destinazione e verificare la copia.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Navigare nella cartella di destinazione e verificare la copia (assert).</t>
         </is>
       </c>
       <c r="G20" s="37" t="inlineStr">
@@ -2657,8 +2657,8 @@
 3. Attendere la ricezione del messaggio.
 4. Inserire il testo univoco nella barra di ricerca.
 5. Avviare la ricerca.
-6. Verificare che il messaggio cercato appaia nei risultati.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il messaggio cercato appaia nei risultati (assert).</t>
         </is>
       </c>
       <c r="G21" s="43" t="inlineStr">
@@ -2698,8 +2698,8 @@
 3. Individuare il pulsante/dropdown filtri.
 4. Cliccare sul filtro per aprire le opzioni.
 5. Selezionare un'opzione di filtro (es. 'Non letti').
-6. Verificare che la lista messaggi sia filtrata correttamente.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che la lista messaggi sia filtrata correttamente (assert).</t>
         </is>
       </c>
       <c r="G22" s="37" t="inlineStr">
@@ -2740,8 +2740,8 @@
 4. Aggiungere un destinatario in CC.
 5. Inserire oggetto e corpo del messaggio.
 6. Cliccare 'Invia'.
-7. Verificare la conferma di invio.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la conferma di invio (assert).</t>
         </is>
       </c>
       <c r="G23" s="43" t="inlineStr">
@@ -2783,8 +2783,8 @@
 5. Cliccare sul pulsante di download dell'allegato.
 6. Gestire il download tramite Playwright expect_download.
 7. Salvare il file nella cartella test-results.
-8. Verificare che il file scaricato esista e abbia dimensione &gt; 0.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che il file scaricato esista e abbia dimensione &gt; 0 (assert).</t>
         </is>
       </c>
       <c r="G24" s="37" t="inlineStr">
@@ -2866,8 +2866,8 @@
 3. Attendere la conferma di invio.
 4. Navigare nella cartella Inviati.
 5. Cercare il messaggio con l'oggetto univoco.
-6. Verificare che il messaggio sia presente con il corretto oggetto.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il messaggio sia presente con il corretto oggetto (assert).</t>
         </is>
       </c>
       <c r="G26" s="37" t="inlineStr">
@@ -2908,8 +2908,8 @@
 4. Attendere l'arrivo della Ricevuta di Accettazione (15+ secondi).
 5. Aggiornare la vista messaggi.
 6. Cercare il messaggio con prefisso 'ACCETTAZIONE'.
-7. Verificare la presenza della RA.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la presenza della RA (assert).</t>
         </is>
       </c>
       <c r="G27" s="43" t="inlineStr">
@@ -2950,8 +2950,8 @@
 4. Attendere l'arrivo della Ricevuta di Consegna (25+ secondi).
 5. Aggiornare la vista messaggi.
 6. Cercare il messaggio con prefisso 'CONSEGNA'.
-7. Verificare la presenza della RD.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la presenza della RD (assert).</t>
         </is>
       </c>
       <c r="G28" s="37" t="inlineStr">
@@ -3034,8 +3034,8 @@
 4. Passare il mouse sulla prima riga messaggio per rivelare il checkbox.
 5. Selezionare il checkbox della prima riga.
 6. Passare il mouse sulla seconda riga e selezionare il suo checkbox.
-7. Verificare la comparsa della toolbar azioni batch (Elimina, Segna, ecc.).
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la comparsa della toolbar azioni batch (Elimina, Segna, ecc., assert).</t>
         </is>
       </c>
       <c r="G30" s="37" t="inlineStr">
@@ -3076,8 +3076,8 @@
 4. Inserire oggetto e corpo del messaggio.
 5. Inviare il messaggio.
 6. Attendere la ricezione della notifica di anomalia.
-7. Verificare la presenza della notifica nell'inbox o come avviso UI.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la presenza della notifica nell'inbox o come avviso UI (assert).</t>
         </is>
       </c>
       <c r="G31" s="43" t="inlineStr">
@@ -3119,8 +3119,8 @@
 5. Abilitare la ricorrenza e configurare la regola (es. settimanale).
 6. Salvare l'evento.
 7. Verificare la presenza dell'evento ricorrente nel calendario.
-8. Eliminare l'evento (singolo o tutti).
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare l'evento (singolo o tutti, cleanup).</t>
         </is>
       </c>
       <c r="G32" s="50" t="inlineStr">
@@ -3164,8 +3164,8 @@
 7. Modificare il titolo con uno nuovo.
 8. Salvare la modifica.
 9. Verificare che il nuovo titolo sia visibile nel calendario.
-10. Eliminare l'evento.
-11. Scattare screenshot.</t>
+10. Scattare screenshot.
+11. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
       <c r="G33" s="37" t="inlineStr">
@@ -3206,8 +3206,8 @@
 4. Aggiungere un partecipante come invitato.
 5. Salvare e inviare l'invito.
 6. Navigare in In arrivo messaggi.
-7. Verificare l'arrivo dell'invito come messaggio PEC.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare l'arrivo dell'invito come messaggio PEC (assert).</t>
         </is>
       </c>
       <c r="G34" s="50" t="inlineStr">
@@ -3249,8 +3249,8 @@
 5. Selezionare il file ICS tramite il file picker.
 6. Confermare l'importazione.
 7. Tentare l'esportazione del calendario (via pulsante o menu contestuale).
-8. Eliminare gli eventi importati.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare gli eventi importati (cleanup).</t>
         </is>
       </c>
       <c r="G35" s="37" t="inlineStr">
@@ -3292,8 +3292,8 @@
 5. Confermare la creazione.
 6. Verificare la comparsa del toast di conferma.
 7. Verificare che il nuovo calendario sia visibile nella sidebar.
-8. Eliminare il calendario creato.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare il calendario creato (cleanup).</t>
         </is>
       </c>
       <c r="G36" s="50" t="inlineStr">
@@ -3377,8 +3377,8 @@
 4. Cliccare il pulsante 'Successivo' (&gt;).
 5. Verificare che l'header sia cambiato rispetto al valore iniziale.
 6. Cliccare il pulsante 'Precedente' (&lt;).
-7. Verificare il ritorno al periodo iniziale.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare il ritorno al periodo iniziale (assert).</t>
         </is>
       </c>
       <c r="G38" s="50" t="inlineStr">
@@ -3420,8 +3420,8 @@
 5. Abilitare il toggle/checkbox 'Giornata intera'.
 6. Salvare l'evento.
 7. Verificare la presenza dell'evento nel calendario come evento giornaliero.
-8. Eliminare l'evento.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
       <c r="G39" s="37" t="inlineStr">
@@ -3464,8 +3464,8 @@
 6. Salvare l'evento.
 7. Riaprire l'evento.
 8. Verificare che il promemoria sia presente e configurato.
-9. Eliminare l'evento.
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
       <c r="G40" s="50" t="inlineStr">
@@ -3508,8 +3508,8 @@
 6. Inserire il titolo univoco dell'evento.
 7. Avviare la ricerca.
 8. Verificare che l'evento sia trovato nei risultati.
-9. Eliminare l'evento.
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
       <c r="G41" s="37" t="inlineStr">
@@ -3550,8 +3550,8 @@
 4. Inserire nome, cognome e indirizzo email.
 5. Salvare il contatto.
 6. Verificare la presenza del contatto nella rubrica.
-7. Eliminare il contatto.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Eliminare il contatto (cleanup).</t>
         </is>
       </c>
       <c r="G42" s="57" t="inlineStr">
@@ -3593,8 +3593,8 @@
 5. Salvare il gruppo.
 6. Aggiungere uno o più contatti al gruppo.
 7. Verificare che il gruppo sia visibile nella sidebar.
-8. Verificare che i contatti siano nel gruppo.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che i contatti siano nel gruppo (assert).</t>
         </is>
       </c>
       <c r="G43" s="37" t="inlineStr">
@@ -3635,8 +3635,8 @@
 4. Selezionare 'Esporta' o 'Esporta come CSV'.
 5. Gestire il download del file tramite Playwright expect_download.
 6. Verificare che il file CSV sia scaricato.
-7. Verificare che il file abbia dimensione &gt; 0.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare che il file abbia dimensione &gt; 0 (assert).</t>
         </is>
       </c>
       <c r="G44" s="57" t="inlineStr">
@@ -3678,8 +3678,8 @@
 5. Selezionare il file CSV di test tramite il file picker.
 6. Confermare l'importazione.
 7. Verificare il messaggio di successo.
-8. Verificare che i contatti importati siano nella rubrica.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che i contatti importati siano nella rubrica (assert).</t>
         </is>
       </c>
       <c r="G45" s="37" t="inlineStr">
@@ -3722,8 +3722,8 @@
 6. Cambiare il cognome con un valore nuovo univoco.
 7. Salvare le modifiche.
 8. Cercare il contatto con il nuovo cognome.
-9. Verificare che il contatto sia trovato con i dati aggiornati.
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Verificare che il contatto sia trovato con i dati aggiornati (assert).</t>
         </is>
       </c>
       <c r="G46" s="57" t="inlineStr">
@@ -3765,8 +3765,8 @@
 5. Cliccare 'Elimina contatto'.
 6. Confermare l'eliminazione.
 7. Cercare il contatto eliminato.
-8. Verificare che non sia più presente nella rubrica.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che non sia più presente nella rubrica (assert).</t>
         </is>
       </c>
       <c r="G47" s="37" t="inlineStr">
@@ -3807,8 +3807,8 @@
 4. Inserire il nome univoco nella barra di ricerca.
 5. Avviare la ricerca.
 6. Verificare che il contatto cercato sia nei risultati.
-7. Eliminare il contatto.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Eliminare il contatto (cleanup).</t>
         </is>
       </c>
       <c r="G48" s="57" t="inlineStr">
@@ -3849,8 +3849,8 @@
 4. Cliccare il pulsante stella (preferito).
 5. Navigare nella sezione 'Contatti preferiti' nella sidebar.
 6. Verificare che il contatto sia presente nella sezione Preferiti.
-7. Rimuovere il contatto dai preferiti.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Rimuovere il contatto dai preferiti (cleanup).</t>
         </is>
       </c>
       <c r="G49" s="37" t="inlineStr">
@@ -3890,8 +3890,8 @@
 3. Selezionare un contatto dalla rubrica.
 4. Cliccare il pulsante 'Scrivi email' o 'Invia email'.
 5. Verificare che la finestra di composizione si apra.
-6. Verificare che il campo destinatario sia pre-compilato con l'email del contatto.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il campo destinatario sia pre-compilato con l'email del contatto (assert).</t>
         </is>
       </c>
       <c r="G50" s="57" t="inlineStr">
@@ -3933,8 +3933,8 @@
 5. Selezionare il gruppo.
 6. Cliccare 'Elimina gruppo'.
 7. Confermare l'eliminazione.
-8. Verificare che il gruppo non sia più nella sidebar.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che il gruppo non sia più nella sidebar (assert).</t>
         </is>
       </c>
       <c r="G51" s="37" t="inlineStr">
@@ -3976,8 +3976,8 @@
 5. Inserire il testo della firma.
 6. Salvare la firma.
 7. Verificare che la firma sia visibile nell'elenco firme.
-8. Eliminare la firma.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare la firma (cleanup).</t>
         </is>
       </c>
       <c r="G52" s="64" t="inlineStr">
@@ -4019,8 +4019,8 @@
 5. Salvare le impostazioni.
 6. Verificare l'applicazione della modifica.
 7. Selezionare l'opzione 'In basso'.
-8. Verificare l'applicazione.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare l'applicazione (assert).</t>
         </is>
       </c>
       <c r="G53" s="37" t="inlineStr">
@@ -4062,8 +4062,8 @@
 5. Configurare le condizioni della regola (mittente, oggetto, ecc.).
 6. Configurare l'azione (sposta in cartella, elimina, ecc.).
 7. Salvare la regola.
-8. Verificare la presenza della regola nell'elenco.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la presenza della regola nell'elenco (assert).</t>
         </is>
       </c>
       <c r="G54" s="64" t="inlineStr">
@@ -4102,8 +4102,8 @@
 2. Navigare nella sezione Impostazioni.
 3. Aprire la sotto-sezione 'Avvisi e report' o 'Risposta automatica'.
 4. Verificare che la pagina sia caricata correttamente.
-5. Verificare la presenza dei controlli di configurazione.
-6. Scattare screenshot.</t>
+5. Scattare screenshot.
+6. Verificare la presenza dei controlli di configurazione (assert).</t>
         </is>
       </c>
       <c r="G55" s="37" t="inlineStr">
@@ -4144,8 +4144,8 @@
 4. Aggiungere un indirizzo email alla lista di blocco.
 5. Salvare le impostazioni.
 6. Verificare che l'indirizzo sia nella lista di blocco.
-7. Rimuovere l'indirizzo dalla lista.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Rimuovere l'indirizzo dalla lista (cleanup).</t>
         </is>
       </c>
       <c r="G56" s="64" t="inlineStr">
@@ -4186,8 +4186,8 @@
 4. Verificare la presenza delle opzioni di configurazione (svuotamento automatico, ecc.).
 5. Modificare un'impostazione.
 6. Salvare.
-7. Verificare il salvataggio.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare il salvataggio (assert).</t>
         </is>
       </c>
       <c r="G57" s="37" t="inlineStr">
@@ -4227,8 +4227,8 @@
 3. Aprire la sotto-sezione 'Storico accessi' o 'Accessi recenti'.
 4. Verificare che la pagina si carichi correttamente.
 5. Verificare la presenza del pulsante/link per visualizzare lo storico.
-6. Cliccare il pulsante e verificare la visualizzazione della lista accessi.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Cliccare il pulsante e verificare la visualizzazione della lista accessi (assert).</t>
         </is>
       </c>
       <c r="G58" s="64" t="inlineStr">
@@ -4275,8 +4275,8 @@
 10. Salvare con il pulsante primario.
 11. Verificare il toast di conferma salvataggio.
 12. Ricaricare la pagina e verificare che la selezione sia mantenuta.
-13. Cleanup: ripristinare il primo radio button e salvare.
-14. Scattare screenshot.</t>
+13. Scattare screenshot.
+14. Cleanup: ripristinare il primo radio button e salvare.</t>
         </is>
       </c>
       <c r="G59" s="71" t="inlineStr">
@@ -4320,8 +4320,8 @@
 7. Navigare a /new/messages/INBOX.
 8. Aprire la sezione Archivio tramite il menu waffle (9 punti nell'header).
 9. Verificare che il messaggio con l'oggetto univoco sia presente in Archivio.
-10. Fallback: se il waffle non funziona, verificare l'accesso via settings URL.
-11. Scattare screenshot.</t>
+10. Scattare screenshot.
+11. Fallback: se il waffle non funziona, verificare l'accesso via settings URL (assert).</t>
         </is>
       </c>
       <c r="G60" s="37" t="inlineStr">
@@ -4363,8 +4363,8 @@
 5. Cliccare il pulsante 'Da conservare'.
 6. Verificare che l'URL contenga 'CONSERVAZIONE'.
 7. Verificare la presenza di testo informativo sulla conservazione.
-8. Verificare la presenza del link alle Impostazioni.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la presenza del link alle Impostazioni (assert).</t>
         </is>
       </c>
       <c r="G61" s="78" t="inlineStr">
@@ -4406,8 +4406,8 @@
 5. Cercare la voce 'Conservazione' nel dropdown del waffle.
 6. Cliccare la voce (gestire eventuale apertura in nuova tab).
 7. Verificare che la pagina di Conservazione si carichi correttamente.
-8. Fallback: se il waffle non funziona, navigare direttamente alla URL di Conservazione e verificare.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Fallback: se il waffle non funziona, navigare direttamente alla URL di Conservazione e verificare (assert).</t>
         </is>
       </c>
       <c r="G62" s="37" t="inlineStr">
@@ -4452,8 +4452,8 @@
 8. Attendere il file input (#hidden_input) e impostare il file EML di test.
 9. Attendere il messaggio di conferma importazione.
 10. Navigare a 'Fatture ricevute'.
-11. Verificare che sia presente almeno un messaggio con riferimento a SDI o FatturaPA.
-12. Scattare screenshot.</t>
+11. Scattare screenshot.
+12. Verificare che sia presente almeno un messaggio con riferimento a SDI o FatturaPA (assert).</t>
         </is>
       </c>
       <c r="G63" s="85" t="inlineStr">
@@ -4495,8 +4495,8 @@
 5. Navigare direttamente a /new/settings/read-invoices.
 6. Verificare che la pagina si carichi (stato domcontentloaded).
 7. Verificare la presenza dell'h1 o testo 'Leggi fatture'.
-8. Verificare la presenza di contenuto informativo (cassetto fiscale, AdE, ecc.).
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la presenza di contenuto informativo (cassetto fiscale, AdE, ecc., assert).</t>
         </is>
       </c>
       <c r="G64" s="37" t="inlineStr">
@@ -4540,8 +4540,8 @@
 7. Verificare la presenza di almeno 2 pulsanti 'Gestisci'.
 8. Navigare alla sotto-sezione Multiutente PEC e verificare il contenuto.
 9. Tornare alla panoramica e navigare a Supervisore360.
-10. Verificare il contenuto della sezione Supervisore360.
-11. Scattare screenshot.</t>
+10. Scattare screenshot.
+11. Verificare il contenuto della sezione Supervisore360 (assert).</t>
         </is>
       </c>
       <c r="G65" s="92" t="inlineStr">
@@ -4584,8 +4584,8 @@
 6. Cercare e cliccare il pulsante 'Aggiungi' (multi-fallback selectors).
 7. Skip se il pulsante non e' trovato (pytest.skip).
 8. Verificare che il form o dialog si sia aperto con campi input.
-9. Chiudere il form senza inviare (tasto Annulla o Escape).
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Chiudere il form senza inviare (tasto Annulla o Escape).</t>
         </is>
       </c>
       <c r="G66" s="37" t="inlineStr">
@@ -4629,8 +4629,8 @@
 7. Cercare e cliccare il pulsante 'Aggiungi' o 'Nuova delega' (multi-fallback selectors).
 8. Skip se il pulsante non e' trovato (pytest.skip).
 9. Verificare che il form o dialog si sia aperto con campi email/input.
-10. Chiudere il form senza inviare (tasto Annulla o Escape).
-11. Scattare screenshot.</t>
+10. Scattare screenshot.
+11. Chiudere il form senza inviare (tasto Annulla o Escape).</t>
         </is>
       </c>
       <c r="G67" s="92" t="inlineStr">
@@ -4725,8 +4725,8 @@
 3. Cliccare il pulsante dell'account (username).
 4. Cliccare il pulsante 'Esci' dal menu dropdown.
 5. Attendere il reindirizzamento alla pagina di login.
-6. Verificare che il campo username sia visibile.
-7. Scattare screenshot della pagina di login.</t>
+6. Scattare screenshot della pagina di login.
+7. Verificare che il campo username sia visibile (assert).</t>
         </is>
       </c>
       <c r="E3" s="31" t="inlineStr">
@@ -4760,8 +4760,8 @@
 5. Cliccare il pulsante Login.
 6. Attendere 2 secondi.
 7. Verificare che l'URL non contenga 'INBOX'.
-8. Verificare la visibilità del messaggio di errore.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la visibilità del messaggio di errore (assert).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">
@@ -4860,8 +4860,8 @@
 6. Inviare il messaggio.
 7. Attendere la ricezione nella cartella In arrivo.
 8. Aprire il messaggio ricevuto.
-9. Verificare la presenza dell'allegato nel messaggio.
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Verificare la presenza dell'allegato nel messaggio (assert).</t>
         </is>
       </c>
       <c r="E3" s="43" t="inlineStr">
@@ -4895,8 +4895,8 @@
 5. Cliccare il pulsante 'Inoltra'.
 6. Inserire il destinatario dell'inoltro.
 7. Inviare il messaggio inoltrato.
-8. Verificare la comparsa del toast di conferma.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la comparsa del toast di conferma (assert).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">
@@ -4962,8 +4962,8 @@
 3. Selezionare il file da importare.
 4. Avviare il processo di importazione.
 5. Attendere il completamento dell'importazione.
-6. Verificare il messaggio di conferma.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare il messaggio di conferma (assert).</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
@@ -4996,8 +4996,8 @@
 4. Rinominare la cartella con un nuovo nome.
 5. Verificare il toast di conferma della modifica.
 6. Eliminare la cartella.
-7. Verificare il toast di conferma dell'eliminazione.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare il toast di conferma dell'eliminazione (assert).</t>
         </is>
       </c>
       <c r="E7" s="43" t="inlineStr">
@@ -5030,8 +5030,8 @@
 4. Selezionare il/i messaggio/i da ripristinare.
 5. Cliccare 'Ripristina' o 'Sposta in In arrivo'.
 6. Verificare che i messaggi non siano più nel cestino.
-7. Navigare in In arrivo e verificare la presenza dei messaggi.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Navigare in In arrivo e verificare la presenza dei messaggi (assert).</t>
         </is>
       </c>
       <c r="E8" s="37" t="inlineStr">
@@ -5063,8 +5063,8 @@
 3. Aggiungere il messaggio ai preferiti (stella).
 4. Verificare che il messaggio compaia nella cartella Preferiti/Speciali.
 5. Selezionare un messaggio e cliccare 'Pinna messaggio'.
-6. Verificare la presenza del messaggio pinnato.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare la presenza del messaggio pinnato (assert).</t>
         </is>
       </c>
       <c r="E9" s="43" t="inlineStr">
@@ -5097,8 +5097,8 @@
 4. Tornare in In arrivo e selezionare un messaggio.
 5. Applicare l'etichetta appena creata al messaggio.
 6. Verificare che l'etichetta sia visibile sul messaggio.
-7. Eliminare l'etichetta.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Eliminare l'etichetta (cleanup).</t>
         </is>
       </c>
       <c r="E10" s="37" t="inlineStr">
@@ -5130,8 +5130,8 @@
 3. Cliccare 'Segna come letto'.
 4. Verificare che il messaggio non sia più in grassetto (letto).
 5. Cliccare 'Segna come da leggere' sullo stesso messaggio.
-6. Verificare che il messaggio torni in grassetto (non letto).
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il messaggio torni in grassetto (non letto, assert).</t>
         </is>
       </c>
       <c r="E11" s="43" t="inlineStr">
@@ -5165,8 +5165,8 @@
 5. Inviare il messaggio.
 6. Attendere la ricezione in In arrivo.
 7. Aprire il messaggio ricevuto.
-8. Verificare la presenza dell'indicatore di alta priorità.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la presenza dell'indicatore di alta priorità (assert).</t>
         </is>
       </c>
       <c r="E12" s="37" t="inlineStr">
@@ -5232,8 +5232,8 @@
 3. Inserire l'indirizzo del destinatario.
 4. Inserire oggetto e corpo del messaggio.
 5. Cliccare 'Invia'.
-6. Verificare la comparsa del toast di conferma invio.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare la comparsa del toast di conferma invio (assert).</t>
         </is>
       </c>
       <c r="E14" s="37" t="inlineStr">
@@ -5300,8 +5300,8 @@
 3. Attendere la ricezione del messaggio.
 4. Selezionare il messaggio e cliccare 'Elimina'.
 5. Navigare nella cartella Cestino.
-6. Verificare che il messaggio eliminato sia presente nel cestino.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il messaggio eliminato sia presente nel cestino (assert).</t>
         </is>
       </c>
       <c r="E16" s="37" t="inlineStr">
@@ -5335,8 +5335,8 @@
 5. Selezionare il messaggio e cliccare 'Sposta in...'.
 6. Selezionare la cartella di destinazione.
 7. Verificare che il messaggio non sia più in In arrivo.
-8. Navigare nella cartella di destinazione e verificare la presenza del messaggio.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Navigare nella cartella di destinazione e verificare la presenza del messaggio (assert).</t>
         </is>
       </c>
       <c r="E17" s="43" t="inlineStr">
@@ -5369,8 +5369,8 @@
 4. Selezionare 'Copia in...' dal menu azioni.
 5. Selezionare la cartella di destinazione.
 6. Verificare che il messaggio originale sia ancora in In arrivo.
-7. Navigare nella cartella di destinazione e verificare la copia.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Navigare nella cartella di destinazione e verificare la copia (assert).</t>
         </is>
       </c>
       <c r="E18" s="37" t="inlineStr">
@@ -5402,8 +5402,8 @@
 3. Attendere la ricezione del messaggio.
 4. Inserire il testo univoco nella barra di ricerca.
 5. Avviare la ricerca.
-6. Verificare che il messaggio cercato appaia nei risultati.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il messaggio cercato appaia nei risultati (assert).</t>
         </is>
       </c>
       <c r="E19" s="43" t="inlineStr">
@@ -5435,8 +5435,8 @@
 3. Individuare il pulsante/dropdown filtri.
 4. Cliccare sul filtro per aprire le opzioni.
 5. Selezionare un'opzione di filtro (es. 'Non letti').
-6. Verificare che la lista messaggi sia filtrata correttamente.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che la lista messaggi sia filtrata correttamente (assert).</t>
         </is>
       </c>
       <c r="E20" s="37" t="inlineStr">
@@ -5469,8 +5469,8 @@
 4. Aggiungere un destinatario in CC.
 5. Inserire oggetto e corpo del messaggio.
 6. Cliccare 'Invia'.
-7. Verificare la conferma di invio.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la conferma di invio (assert).</t>
         </is>
       </c>
       <c r="E21" s="43" t="inlineStr">
@@ -5504,8 +5504,8 @@
 5. Cliccare sul pulsante di download dell'allegato.
 6. Gestire il download tramite Playwright expect_download.
 7. Salvare il file nella cartella test-results.
-8. Verificare che il file scaricato esista e abbia dimensione &gt; 0.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che il file scaricato esista e abbia dimensione &gt; 0 (assert).</t>
         </is>
       </c>
       <c r="E22" s="37" t="inlineStr">
@@ -5571,8 +5571,8 @@
 3. Attendere la conferma di invio.
 4. Navigare nella cartella Inviati.
 5. Cercare il messaggio con l'oggetto univoco.
-6. Verificare che il messaggio sia presente con il corretto oggetto.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il messaggio sia presente con il corretto oggetto (assert).</t>
         </is>
       </c>
       <c r="E24" s="37" t="inlineStr">
@@ -5605,8 +5605,8 @@
 4. Attendere l'arrivo della Ricevuta di Accettazione (15+ secondi).
 5. Aggiornare la vista messaggi.
 6. Cercare il messaggio con prefisso 'ACCETTAZIONE'.
-7. Verificare la presenza della RA.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la presenza della RA (assert).</t>
         </is>
       </c>
       <c r="E25" s="43" t="inlineStr">
@@ -5639,8 +5639,8 @@
 4. Attendere l'arrivo della Ricevuta di Consegna (25+ secondi).
 5. Aggiornare la vista messaggi.
 6. Cercare il messaggio con prefisso 'CONSEGNA'.
-7. Verificare la presenza della RD.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la presenza della RD (assert).</t>
         </is>
       </c>
       <c r="E26" s="37" t="inlineStr">
@@ -5707,8 +5707,8 @@
 4. Passare il mouse sulla prima riga messaggio per rivelare il checkbox.
 5. Selezionare il checkbox della prima riga.
 6. Passare il mouse sulla seconda riga e selezionare il suo checkbox.
-7. Verificare la comparsa della toolbar azioni batch (Elimina, Segna, ecc.).
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la comparsa della toolbar azioni batch (Elimina, Segna, ecc., assert).</t>
         </is>
       </c>
       <c r="E28" s="37" t="inlineStr">
@@ -5741,8 +5741,8 @@
 4. Inserire oggetto e corpo del messaggio.
 5. Inviare il messaggio.
 6. Attendere la ricezione della notifica di anomalia.
-7. Verificare la presenza della notifica nell'inbox o come avviso UI.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare la presenza della notifica nell'inbox o come avviso UI (assert).</t>
         </is>
       </c>
       <c r="E29" s="43" t="inlineStr">
@@ -5840,8 +5840,8 @@
 5. Abilitare la ricorrenza e configurare la regola (es. settimanale).
 6. Salvare l'evento.
 7. Verificare la presenza dell'evento ricorrente nel calendario.
-8. Eliminare l'evento (singolo o tutti).
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare l'evento (singolo o tutti, cleanup).</t>
         </is>
       </c>
       <c r="E3" s="50" t="inlineStr">
@@ -5877,8 +5877,8 @@
 7. Modificare il titolo con uno nuovo.
 8. Salvare la modifica.
 9. Verificare che il nuovo titolo sia visibile nel calendario.
-10. Eliminare l'evento.
-11. Scattare screenshot.</t>
+10. Scattare screenshot.
+11. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">
@@ -5911,8 +5911,8 @@
 4. Aggiungere un partecipante come invitato.
 5. Salvare e inviare l'invito.
 6. Navigare in In arrivo messaggi.
-7. Verificare l'arrivo dell'invito come messaggio PEC.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare l'arrivo dell'invito come messaggio PEC (assert).</t>
         </is>
       </c>
       <c r="E5" s="50" t="inlineStr">
@@ -5946,8 +5946,8 @@
 5. Selezionare il file ICS tramite il file picker.
 6. Confermare l'importazione.
 7. Tentare l'esportazione del calendario (via pulsante o menu contestuale).
-8. Eliminare gli eventi importati.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare gli eventi importati (cleanup).</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
@@ -5981,8 +5981,8 @@
 5. Confermare la creazione.
 6. Verificare la comparsa del toast di conferma.
 7. Verificare che il nuovo calendario sia visibile nella sidebar.
-8. Eliminare il calendario creato.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare il calendario creato (cleanup).</t>
         </is>
       </c>
       <c r="E7" s="50" t="inlineStr">
@@ -6050,8 +6050,8 @@
 4. Cliccare il pulsante 'Successivo' (&gt;).
 5. Verificare che l'header sia cambiato rispetto al valore iniziale.
 6. Cliccare il pulsante 'Precedente' (&lt;).
-7. Verificare il ritorno al periodo iniziale.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare il ritorno al periodo iniziale (assert).</t>
         </is>
       </c>
       <c r="E9" s="50" t="inlineStr">
@@ -6085,8 +6085,8 @@
 5. Abilitare il toggle/checkbox 'Giornata intera'.
 6. Salvare l'evento.
 7. Verificare la presenza dell'evento nel calendario come evento giornaliero.
-8. Eliminare l'evento.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
       <c r="E10" s="37" t="inlineStr">
@@ -6121,8 +6121,8 @@
 6. Salvare l'evento.
 7. Riaprire l'evento.
 8. Verificare che il promemoria sia presente e configurato.
-9. Eliminare l'evento.
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
       <c r="E11" s="50" t="inlineStr">
@@ -6157,8 +6157,8 @@
 6. Inserire il titolo univoco dell'evento.
 7. Avviare la ricerca.
 8. Verificare che l'evento sia trovato nei risultati.
-9. Eliminare l'evento.
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Eliminare l'evento (cleanup).</t>
         </is>
       </c>
       <c r="E12" s="37" t="inlineStr">
@@ -6255,8 +6255,8 @@
 4. Inserire nome, cognome e indirizzo email.
 5. Salvare il contatto.
 6. Verificare la presenza del contatto nella rubrica.
-7. Eliminare il contatto.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Eliminare il contatto (cleanup).</t>
         </is>
       </c>
       <c r="E3" s="57" t="inlineStr">
@@ -6290,8 +6290,8 @@
 5. Salvare il gruppo.
 6. Aggiungere uno o più contatti al gruppo.
 7. Verificare che il gruppo sia visibile nella sidebar.
-8. Verificare che i contatti siano nel gruppo.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che i contatti siano nel gruppo (assert).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">
@@ -6324,8 +6324,8 @@
 4. Selezionare 'Esporta' o 'Esporta come CSV'.
 5. Gestire il download del file tramite Playwright expect_download.
 6. Verificare che il file CSV sia scaricato.
-7. Verificare che il file abbia dimensione &gt; 0.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare che il file abbia dimensione &gt; 0 (assert).</t>
         </is>
       </c>
       <c r="E5" s="57" t="inlineStr">
@@ -6359,8 +6359,8 @@
 5. Selezionare il file CSV di test tramite il file picker.
 6. Confermare l'importazione.
 7. Verificare il messaggio di successo.
-8. Verificare che i contatti importati siano nella rubrica.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che i contatti importati siano nella rubrica (assert).</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
@@ -6395,8 +6395,8 @@
 6. Cambiare il cognome con un valore nuovo univoco.
 7. Salvare le modifiche.
 8. Cercare il contatto con il nuovo cognome.
-9. Verificare che il contatto sia trovato con i dati aggiornati.
-10. Scattare screenshot.</t>
+9. Scattare screenshot.
+10. Verificare che il contatto sia trovato con i dati aggiornati (assert).</t>
         </is>
       </c>
       <c r="E7" s="57" t="inlineStr">
@@ -6430,8 +6430,8 @@
 5. Cliccare 'Elimina contatto'.
 6. Confermare l'eliminazione.
 7. Cercare il contatto eliminato.
-8. Verificare che non sia più presente nella rubrica.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che non sia più presente nella rubrica (assert).</t>
         </is>
       </c>
       <c r="E8" s="37" t="inlineStr">
@@ -6464,8 +6464,8 @@
 4. Inserire il nome univoco nella barra di ricerca.
 5. Avviare la ricerca.
 6. Verificare che il contatto cercato sia nei risultati.
-7. Eliminare il contatto.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Eliminare il contatto (cleanup).</t>
         </is>
       </c>
       <c r="E9" s="57" t="inlineStr">
@@ -6498,8 +6498,8 @@
 4. Cliccare il pulsante stella (preferito).
 5. Navigare nella sezione 'Contatti preferiti' nella sidebar.
 6. Verificare che il contatto sia presente nella sezione Preferiti.
-7. Rimuovere il contatto dai preferiti.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Rimuovere il contatto dai preferiti (cleanup).</t>
         </is>
       </c>
       <c r="E10" s="37" t="inlineStr">
@@ -6531,8 +6531,8 @@
 3. Selezionare un contatto dalla rubrica.
 4. Cliccare il pulsante 'Scrivi email' o 'Invia email'.
 5. Verificare che la finestra di composizione si apra.
-6. Verificare che il campo destinatario sia pre-compilato con l'email del contatto.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Verificare che il campo destinatario sia pre-compilato con l'email del contatto (assert).</t>
         </is>
       </c>
       <c r="E11" s="57" t="inlineStr">
@@ -6566,8 +6566,8 @@
 5. Selezionare il gruppo.
 6. Cliccare 'Elimina gruppo'.
 7. Confermare l'eliminazione.
-8. Verificare che il gruppo non sia più nella sidebar.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare che il gruppo non sia più nella sidebar (assert).</t>
         </is>
       </c>
       <c r="E12" s="37" t="inlineStr">
@@ -6665,8 +6665,8 @@
 5. Inserire il testo della firma.
 6. Salvare la firma.
 7. Verificare che la firma sia visibile nell'elenco firme.
-8. Eliminare la firma.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Eliminare la firma (cleanup).</t>
         </is>
       </c>
       <c r="E3" s="64" t="inlineStr">
@@ -6700,8 +6700,8 @@
 5. Salvare le impostazioni.
 6. Verificare l'applicazione della modifica.
 7. Selezionare l'opzione 'In basso'.
-8. Verificare l'applicazione.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare l'applicazione (assert).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">
@@ -6735,8 +6735,8 @@
 5. Configurare le condizioni della regola (mittente, oggetto, ecc.).
 6. Configurare l'azione (sposta in cartella, elimina, ecc.).
 7. Salvare la regola.
-8. Verificare la presenza della regola nell'elenco.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la presenza della regola nell'elenco (assert).</t>
         </is>
       </c>
       <c r="E5" s="64" t="inlineStr">
@@ -6767,8 +6767,8 @@
 2. Navigare nella sezione Impostazioni.
 3. Aprire la sotto-sezione 'Avvisi e report' o 'Risposta automatica'.
 4. Verificare che la pagina sia caricata correttamente.
-5. Verificare la presenza dei controlli di configurazione.
-6. Scattare screenshot.</t>
+5. Scattare screenshot.
+6. Verificare la presenza dei controlli di configurazione (assert).</t>
         </is>
       </c>
       <c r="E6" s="37" t="inlineStr">
@@ -6801,8 +6801,8 @@
 4. Aggiungere un indirizzo email alla lista di blocco.
 5. Salvare le impostazioni.
 6. Verificare che l'indirizzo sia nella lista di blocco.
-7. Rimuovere l'indirizzo dalla lista.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Rimuovere l'indirizzo dalla lista (cleanup).</t>
         </is>
       </c>
       <c r="E7" s="64" t="inlineStr">
@@ -6835,8 +6835,8 @@
 4. Verificare la presenza delle opzioni di configurazione (svuotamento automatico, ecc.).
 5. Modificare un'impostazione.
 6. Salvare.
-7. Verificare il salvataggio.
-8. Scattare screenshot.</t>
+7. Scattare screenshot.
+8. Verificare il salvataggio (assert).</t>
         </is>
       </c>
       <c r="E8" s="37" t="inlineStr">
@@ -6868,8 +6868,8 @@
 3. Aprire la sotto-sezione 'Storico accessi' o 'Accessi recenti'.
 4. Verificare che la pagina si carichi correttamente.
 5. Verificare la presenza del pulsante/link per visualizzare lo storico.
-6. Cliccare il pulsante e verificare la visualizzazione della lista accessi.
-7. Scattare screenshot.</t>
+6. Scattare screenshot.
+7. Cliccare il pulsante e verificare la visualizzazione della lista accessi (assert).</t>
         </is>
       </c>
       <c r="E9" s="64" t="inlineStr">
@@ -6972,8 +6972,8 @@
 10. Salvare con il pulsante primario.
 11. Verificare il toast di conferma salvataggio.
 12. Ricaricare la pagina e verificare che la selezione sia mantenuta.
-13. Cleanup: ripristinare il primo radio button e salvare.
-14. Scattare screenshot.</t>
+13. Scattare screenshot.
+14. Cleanup: ripristinare il primo radio button e salvare.</t>
         </is>
       </c>
       <c r="E3" s="71" t="inlineStr">
@@ -7009,8 +7009,8 @@
 7. Navigare a /new/messages/INBOX.
 8. Aprire la sezione Archivio tramite il menu waffle (9 punti nell'header).
 9. Verificare che il messaggio con l'oggetto univoco sia presente in Archivio.
-10. Fallback: se il waffle non funziona, verificare l'accesso via settings URL.
-11. Scattare screenshot.</t>
+10. Scattare screenshot.
+11. Fallback: se il waffle non funziona, verificare l'accesso via settings URL (assert).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">
@@ -7108,8 +7108,8 @@
 5. Cliccare il pulsante 'Da conservare'.
 6. Verificare che l'URL contenga 'CONSERVAZIONE'.
 7. Verificare la presenza di testo informativo sulla conservazione.
-8. Verificare la presenza del link alle Impostazioni.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Verificare la presenza del link alle Impostazioni (assert).</t>
         </is>
       </c>
       <c r="E3" s="78" t="inlineStr">
@@ -7143,8 +7143,8 @@
 5. Cercare la voce 'Conservazione' nel dropdown del waffle.
 6. Cliccare la voce (gestire eventuale apertura in nuova tab).
 7. Verificare che la pagina di Conservazione si carichi correttamente.
-8. Fallback: se il waffle non funziona, navigare direttamente alla URL di Conservazione e verificare.
-9. Scattare screenshot.</t>
+8. Scattare screenshot.
+9. Fallback: se il waffle non funziona, navigare direttamente alla URL di Conservazione e verificare (assert).</t>
         </is>
       </c>
       <c r="E4" s="37" t="inlineStr">

</xml_diff>

<commit_message>
fix(mobile/archivio): login mobile e altezza righe Excel
- base_mobile.py: aggiunto wait_for_url INBOX nel blocco smart-login
  per evitare falso re-login su redirect auth→INBOX (10/10 test passati)
- test_archivio_01/02.py: rimossi except:pass su step funzionali critici
  post-skip; wait_for_load_state sostituito con wait_for_timeout
- genera_excel_suite.py + suite_test_pec.xlsx: altezza righe calcolata
  considerando il wrapping automatico del testo per colonna

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/suite_test_pec.xlsx
+++ b/suite_test_pec.xlsx
@@ -1552,7 +1552,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="168" customHeight="1">
+    <row r="3" ht="224" customHeight="1">
       <c r="A3" s="156" t="n">
         <v>61</v>
       </c>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="F3" s="160" t="inlineStr"/>
     </row>
-    <row r="4" ht="126" customHeight="1">
+    <row r="4" ht="168" customHeight="1">
       <c r="A4" s="161" t="n">
         <v>62</v>
       </c>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="154" customHeight="1">
+    <row r="3" ht="224" customHeight="1">
       <c r="A3" s="164" t="n">
         <v>63</v>
       </c>
@@ -1726,7 +1726,7 @@
       </c>
       <c r="F3" s="168" t="inlineStr"/>
     </row>
-    <row r="4" ht="140" customHeight="1">
+    <row r="4" ht="210" customHeight="1">
       <c r="A4" s="169" t="n">
         <v>64</v>
       </c>
@@ -1762,7 +1762,7 @@
       </c>
       <c r="F4" s="105" t="inlineStr"/>
     </row>
-    <row r="5" ht="154" customHeight="1">
+    <row r="5" ht="210" customHeight="1">
       <c r="A5" s="164" t="n">
         <v>65</v>
       </c>
@@ -1869,7 +1869,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98" customHeight="1">
+    <row r="3" ht="126" customHeight="1">
       <c r="A3" s="26" t="n">
         <v>1</v>
       </c>
@@ -1910,7 +1910,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="126" customHeight="1">
+    <row r="4" ht="168" customHeight="1">
       <c r="A4" s="32" t="n">
         <v>2</v>
       </c>
@@ -1953,7 +1953,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="140" customHeight="1">
+    <row r="5" ht="196" customHeight="1">
       <c r="A5" s="38" t="n">
         <v>3</v>
       </c>
@@ -1997,7 +1997,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="126" customHeight="1">
+    <row r="6" ht="154" customHeight="1">
       <c r="A6" s="44" t="n">
         <v>4</v>
       </c>
@@ -2040,7 +2040,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="112" customHeight="1">
+    <row r="7" ht="126" customHeight="1">
       <c r="A7" s="38" t="n">
         <v>5</v>
       </c>
@@ -2123,7 +2123,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="112" customHeight="1">
+    <row r="9" ht="154" customHeight="1">
       <c r="A9" s="38" t="n">
         <v>7</v>
       </c>
@@ -2165,7 +2165,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="112" customHeight="1">
+    <row r="10" ht="140" customHeight="1">
       <c r="A10" s="44" t="n">
         <v>8</v>
       </c>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="98" customHeight="1">
+    <row r="11" ht="140" customHeight="1">
       <c r="A11" s="38" t="n">
         <v>9</v>
       </c>
@@ -2248,7 +2248,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="112" customHeight="1">
+    <row r="12" ht="168" customHeight="1">
       <c r="A12" s="44" t="n">
         <v>10</v>
       </c>
@@ -2290,7 +2290,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="98" customHeight="1">
+    <row r="13" ht="154" customHeight="1">
       <c r="A13" s="38" t="n">
         <v>11</v>
       </c>
@@ -2331,7 +2331,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="126" customHeight="1">
+    <row r="14" ht="140" customHeight="1">
       <c r="A14" s="44" t="n">
         <v>12</v>
       </c>
@@ -2374,7 +2374,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="112" customHeight="1">
+    <row r="15" ht="126" customHeight="1">
       <c r="A15" s="38" t="n">
         <v>13</v>
       </c>
@@ -2416,7 +2416,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="98" customHeight="1">
+    <row r="16" ht="112" customHeight="1">
       <c r="A16" s="44" t="n">
         <v>14</v>
       </c>
@@ -2457,7 +2457,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="126" customHeight="1">
+    <row r="17" ht="154" customHeight="1">
       <c r="A17" s="38" t="n">
         <v>15</v>
       </c>
@@ -2500,7 +2500,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="98" customHeight="1">
+    <row r="18" ht="126" customHeight="1">
       <c r="A18" s="44" t="n">
         <v>16</v>
       </c>
@@ -2541,7 +2541,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="126" customHeight="1">
+    <row r="19" ht="168" customHeight="1">
       <c r="A19" s="38" t="n">
         <v>17</v>
       </c>
@@ -2584,7 +2584,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="112" customHeight="1">
+    <row r="20" ht="140" customHeight="1">
       <c r="A20" s="44" t="n">
         <v>18</v>
       </c>
@@ -2626,7 +2626,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="98" customHeight="1">
+    <row r="21" ht="140" customHeight="1">
       <c r="A21" s="38" t="n">
         <v>19</v>
       </c>
@@ -2667,7 +2667,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="98" customHeight="1">
+    <row r="22" ht="126" customHeight="1">
       <c r="A22" s="44" t="n">
         <v>20</v>
       </c>
@@ -2708,7 +2708,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="112" customHeight="1">
+    <row r="23" ht="126" customHeight="1">
       <c r="A23" s="38" t="n">
         <v>21</v>
       </c>
@@ -2750,7 +2750,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="126" customHeight="1">
+    <row r="24" ht="182" customHeight="1">
       <c r="A24" s="44" t="n">
         <v>22</v>
       </c>
@@ -2793,7 +2793,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="112" customHeight="1">
+    <row r="25" ht="140" customHeight="1">
       <c r="A25" s="38" t="n">
         <v>23</v>
       </c>
@@ -2835,7 +2835,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="98" customHeight="1">
+    <row r="26" ht="112" customHeight="1">
       <c r="A26" s="44" t="n">
         <v>24</v>
       </c>
@@ -2876,7 +2876,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="112" customHeight="1">
+    <row r="27" ht="154" customHeight="1">
       <c r="A27" s="38" t="n">
         <v>25</v>
       </c>
@@ -2918,7 +2918,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="112" customHeight="1">
+    <row r="28" ht="140" customHeight="1">
       <c r="A28" s="44" t="n">
         <v>26</v>
       </c>
@@ -2960,7 +2960,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="112" customHeight="1">
+    <row r="29" ht="154" customHeight="1">
       <c r="A29" s="38" t="n">
         <v>27</v>
       </c>
@@ -3002,7 +3002,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="112" customHeight="1">
+    <row r="30" ht="182" customHeight="1">
       <c r="A30" s="44" t="n">
         <v>28</v>
       </c>
@@ -3044,7 +3044,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="112" customHeight="1">
+    <row r="31" ht="154" customHeight="1">
       <c r="A31" s="38" t="n">
         <v>29</v>
       </c>
@@ -3086,7 +3086,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="126" customHeight="1">
+    <row r="32" ht="154" customHeight="1">
       <c r="A32" s="45" t="n">
         <v>30</v>
       </c>
@@ -3129,7 +3129,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="154" customHeight="1">
+    <row r="33" ht="168" customHeight="1">
       <c r="A33" s="51" t="n">
         <v>31</v>
       </c>
@@ -3174,7 +3174,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="112" customHeight="1">
+    <row r="34" ht="126" customHeight="1">
       <c r="A34" s="45" t="n">
         <v>32</v>
       </c>
@@ -3216,7 +3216,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="126" customHeight="1">
+    <row r="35" ht="154" customHeight="1">
       <c r="A35" s="51" t="n">
         <v>33</v>
       </c>
@@ -3259,7 +3259,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="126" customHeight="1">
+    <row r="36" ht="168" customHeight="1">
       <c r="A36" s="45" t="n">
         <v>34</v>
       </c>
@@ -3345,7 +3345,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="112" customHeight="1">
+    <row r="38" ht="154" customHeight="1">
       <c r="A38" s="45" t="n">
         <v>36</v>
       </c>
@@ -3387,7 +3387,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="126" customHeight="1">
+    <row r="39" ht="154" customHeight="1">
       <c r="A39" s="51" t="n">
         <v>37</v>
       </c>
@@ -3430,7 +3430,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="140" customHeight="1">
+    <row r="40" ht="168" customHeight="1">
       <c r="A40" s="45" t="n">
         <v>38</v>
       </c>
@@ -3474,7 +3474,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="140" customHeight="1">
+    <row r="41" ht="154" customHeight="1">
       <c r="A41" s="51" t="n">
         <v>39</v>
       </c>
@@ -3518,7 +3518,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="112" customHeight="1">
+    <row r="42" ht="126" customHeight="1">
       <c r="A42" s="52" t="n">
         <v>40</v>
       </c>
@@ -3560,7 +3560,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="126" customHeight="1">
+    <row r="43" ht="154" customHeight="1">
       <c r="A43" s="58" t="n">
         <v>41</v>
       </c>
@@ -3603,7 +3603,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="112" customHeight="1">
+    <row r="44" ht="154" customHeight="1">
       <c r="A44" s="52" t="n">
         <v>42</v>
       </c>
@@ -3645,7 +3645,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="126" customHeight="1">
+    <row r="45" ht="168" customHeight="1">
       <c r="A45" s="58" t="n">
         <v>43</v>
       </c>
@@ -3688,7 +3688,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="140" customHeight="1">
+    <row r="46" ht="168" customHeight="1">
       <c r="A46" s="52" t="n">
         <v>44</v>
       </c>
@@ -3732,7 +3732,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="126" customHeight="1">
+    <row r="47" ht="140" customHeight="1">
       <c r="A47" s="58" t="n">
         <v>45</v>
       </c>
@@ -3775,7 +3775,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="112" customHeight="1">
+    <row r="48" ht="140" customHeight="1">
       <c r="A48" s="52" t="n">
         <v>46</v>
       </c>
@@ -3817,7 +3817,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="112" customHeight="1">
+    <row r="49" ht="140" customHeight="1">
       <c r="A49" s="58" t="n">
         <v>47</v>
       </c>
@@ -3859,7 +3859,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="98" customHeight="1">
+    <row r="50" ht="140" customHeight="1">
       <c r="A50" s="52" t="n">
         <v>48</v>
       </c>
@@ -3900,7 +3900,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="126" customHeight="1">
+    <row r="51" ht="154" customHeight="1">
       <c r="A51" s="58" t="n">
         <v>49</v>
       </c>
@@ -3943,7 +3943,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="126" customHeight="1">
+    <row r="52" ht="140" customHeight="1">
       <c r="A52" s="59" t="n">
         <v>50</v>
       </c>
@@ -4029,7 +4029,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="126" customHeight="1">
+    <row r="54" ht="182" customHeight="1">
       <c r="A54" s="59" t="n">
         <v>52</v>
       </c>
@@ -4072,7 +4072,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="84" customHeight="1">
+    <row r="55" ht="126" customHeight="1">
       <c r="A55" s="65" t="n">
         <v>53</v>
       </c>
@@ -4112,7 +4112,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="112" customHeight="1">
+    <row r="56" ht="140" customHeight="1">
       <c r="A56" s="59" t="n">
         <v>54</v>
       </c>
@@ -4154,7 +4154,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="112" customHeight="1">
+    <row r="57" ht="126" customHeight="1">
       <c r="A57" s="65" t="n">
         <v>55</v>
       </c>
@@ -4196,7 +4196,7 @@
         </is>
       </c>
     </row>
-    <row r="58" ht="98" customHeight="1">
+    <row r="58" ht="154" customHeight="1">
       <c r="A58" s="59" t="n">
         <v>56</v>
       </c>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
     </row>
-    <row r="59" ht="196" customHeight="1">
+    <row r="59" ht="308" customHeight="1">
       <c r="A59" s="66" t="n">
         <v>57</v>
       </c>
@@ -4285,7 +4285,7 @@
         </is>
       </c>
     </row>
-    <row r="60" ht="154" customHeight="1">
+    <row r="60" ht="252" customHeight="1">
       <c r="A60" s="72" t="n">
         <v>58</v>
       </c>
@@ -4330,7 +4330,7 @@
         </is>
       </c>
     </row>
-    <row r="61" ht="126" customHeight="1">
+    <row r="61" ht="168" customHeight="1">
       <c r="A61" s="73" t="n">
         <v>59</v>
       </c>
@@ -4373,7 +4373,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="126" customHeight="1">
+    <row r="62" ht="224" customHeight="1">
       <c r="A62" s="79" t="n">
         <v>60</v>
       </c>
@@ -4416,7 +4416,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="168" customHeight="1">
+    <row r="63" ht="252" customHeight="1">
       <c r="A63" s="80" t="n">
         <v>61</v>
       </c>
@@ -4462,7 +4462,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="126" customHeight="1">
+    <row r="64" ht="196" customHeight="1">
       <c r="A64" s="86" t="n">
         <v>62</v>
       </c>
@@ -4505,7 +4505,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="154" customHeight="1">
+    <row r="65" ht="252" customHeight="1">
       <c r="A65" s="87" t="n">
         <v>63</v>
       </c>
@@ -4550,7 +4550,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="140" customHeight="1">
+    <row r="66" ht="252" customHeight="1">
       <c r="A66" s="93" t="n">
         <v>64</v>
       </c>
@@ -4594,7 +4594,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="154" customHeight="1">
+    <row r="67" ht="266" customHeight="1">
       <c r="A67" s="87" t="n">
         <v>65</v>
       </c>
@@ -4703,7 +4703,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="98" customHeight="1">
+    <row r="3" ht="112" customHeight="1">
       <c r="A3" s="96" t="n">
         <v>1</v>
       </c>
@@ -4736,7 +4736,7 @@
       </c>
       <c r="F3" s="100" t="inlineStr"/>
     </row>
-    <row r="4" ht="126" customHeight="1">
+    <row r="4" ht="140" customHeight="1">
       <c r="A4" s="101" t="n">
         <v>2</v>
       </c>
@@ -4835,7 +4835,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="140" customHeight="1">
+    <row r="3" ht="154" customHeight="1">
       <c r="A3" s="108" t="n">
         <v>3</v>
       </c>
@@ -4906,7 +4906,7 @@
       </c>
       <c r="F4" s="105" t="inlineStr"/>
     </row>
-    <row r="5" ht="112" customHeight="1">
+    <row r="5" ht="126" customHeight="1">
       <c r="A5" s="108" t="n">
         <v>5</v>
       </c>
@@ -4973,7 +4973,7 @@
       </c>
       <c r="F6" s="105" t="inlineStr"/>
     </row>
-    <row r="7" ht="112" customHeight="1">
+    <row r="7" ht="126" customHeight="1">
       <c r="A7" s="108" t="n">
         <v>7</v>
       </c>
@@ -5007,7 +5007,7 @@
       </c>
       <c r="F7" s="112" t="inlineStr"/>
     </row>
-    <row r="8" ht="112" customHeight="1">
+    <row r="8" ht="126" customHeight="1">
       <c r="A8" s="113" t="n">
         <v>8</v>
       </c>
@@ -5041,7 +5041,7 @@
       </c>
       <c r="F8" s="105" t="inlineStr"/>
     </row>
-    <row r="9" ht="98" customHeight="1">
+    <row r="9" ht="112" customHeight="1">
       <c r="A9" s="108" t="n">
         <v>9</v>
       </c>
@@ -5108,7 +5108,7 @@
       </c>
       <c r="F10" s="105" t="inlineStr"/>
     </row>
-    <row r="11" ht="98" customHeight="1">
+    <row r="11" ht="140" customHeight="1">
       <c r="A11" s="108" t="n">
         <v>11</v>
       </c>
@@ -5141,7 +5141,7 @@
       </c>
       <c r="F11" s="112" t="inlineStr"/>
     </row>
-    <row r="12" ht="126" customHeight="1">
+    <row r="12" ht="140" customHeight="1">
       <c r="A12" s="113" t="n">
         <v>12</v>
       </c>
@@ -5176,7 +5176,7 @@
       </c>
       <c r="F12" s="105" t="inlineStr"/>
     </row>
-    <row r="13" ht="112" customHeight="1">
+    <row r="13" ht="126" customHeight="1">
       <c r="A13" s="108" t="n">
         <v>13</v>
       </c>
@@ -5210,7 +5210,7 @@
       </c>
       <c r="F13" s="112" t="inlineStr"/>
     </row>
-    <row r="14" ht="98" customHeight="1">
+    <row r="14" ht="112" customHeight="1">
       <c r="A14" s="113" t="n">
         <v>14</v>
       </c>
@@ -5243,7 +5243,7 @@
       </c>
       <c r="F14" s="105" t="inlineStr"/>
     </row>
-    <row r="15" ht="126" customHeight="1">
+    <row r="15" ht="154" customHeight="1">
       <c r="A15" s="108" t="n">
         <v>15</v>
       </c>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="F15" s="112" t="inlineStr"/>
     </row>
-    <row r="16" ht="98" customHeight="1">
+    <row r="16" ht="112" customHeight="1">
       <c r="A16" s="113" t="n">
         <v>16</v>
       </c>
@@ -5311,7 +5311,7 @@
       </c>
       <c r="F16" s="105" t="inlineStr"/>
     </row>
-    <row r="17" ht="126" customHeight="1">
+    <row r="17" ht="140" customHeight="1">
       <c r="A17" s="108" t="n">
         <v>17</v>
       </c>
@@ -5346,7 +5346,7 @@
       </c>
       <c r="F17" s="112" t="inlineStr"/>
     </row>
-    <row r="18" ht="112" customHeight="1">
+    <row r="18" ht="140" customHeight="1">
       <c r="A18" s="113" t="n">
         <v>18</v>
       </c>
@@ -5380,7 +5380,7 @@
       </c>
       <c r="F18" s="105" t="inlineStr"/>
     </row>
-    <row r="19" ht="98" customHeight="1">
+    <row r="19" ht="112" customHeight="1">
       <c r="A19" s="108" t="n">
         <v>19</v>
       </c>
@@ -5413,7 +5413,7 @@
       </c>
       <c r="F19" s="112" t="inlineStr"/>
     </row>
-    <row r="20" ht="98" customHeight="1">
+    <row r="20" ht="112" customHeight="1">
       <c r="A20" s="113" t="n">
         <v>20</v>
       </c>
@@ -5480,7 +5480,7 @@
       </c>
       <c r="F21" s="112" t="inlineStr"/>
     </row>
-    <row r="22" ht="126" customHeight="1">
+    <row r="22" ht="154" customHeight="1">
       <c r="A22" s="113" t="n">
         <v>22</v>
       </c>
@@ -5549,7 +5549,7 @@
       </c>
       <c r="F23" s="112" t="inlineStr"/>
     </row>
-    <row r="24" ht="98" customHeight="1">
+    <row r="24" ht="112" customHeight="1">
       <c r="A24" s="113" t="n">
         <v>24</v>
       </c>
@@ -5582,7 +5582,7 @@
       </c>
       <c r="F24" s="105" t="inlineStr"/>
     </row>
-    <row r="25" ht="112" customHeight="1">
+    <row r="25" ht="140" customHeight="1">
       <c r="A25" s="108" t="n">
         <v>25</v>
       </c>
@@ -5616,7 +5616,7 @@
       </c>
       <c r="F25" s="112" t="inlineStr"/>
     </row>
-    <row r="26" ht="112" customHeight="1">
+    <row r="26" ht="140" customHeight="1">
       <c r="A26" s="113" t="n">
         <v>26</v>
       </c>
@@ -5650,7 +5650,7 @@
       </c>
       <c r="F26" s="105" t="inlineStr"/>
     </row>
-    <row r="27" ht="112" customHeight="1">
+    <row r="27" ht="154" customHeight="1">
       <c r="A27" s="108" t="n">
         <v>27</v>
       </c>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="F27" s="112" t="inlineStr"/>
     </row>
-    <row r="28" ht="112" customHeight="1">
+    <row r="28" ht="154" customHeight="1">
       <c r="A28" s="113" t="n">
         <v>28</v>
       </c>
@@ -5718,7 +5718,7 @@
       </c>
       <c r="F28" s="105" t="inlineStr"/>
     </row>
-    <row r="29" ht="112" customHeight="1">
+    <row r="29" ht="140" customHeight="1">
       <c r="A29" s="108" t="n">
         <v>29</v>
       </c>
@@ -5816,7 +5816,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="126" customHeight="1">
+    <row r="3" ht="154" customHeight="1">
       <c r="A3" s="116" t="n">
         <v>30</v>
       </c>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="F3" s="120" t="inlineStr"/>
     </row>
-    <row r="4" ht="154" customHeight="1">
+    <row r="4" ht="168" customHeight="1">
       <c r="A4" s="121" t="n">
         <v>31</v>
       </c>
@@ -5888,7 +5888,7 @@
       </c>
       <c r="F4" s="105" t="inlineStr"/>
     </row>
-    <row r="5" ht="112" customHeight="1">
+    <row r="5" ht="126" customHeight="1">
       <c r="A5" s="116" t="n">
         <v>32</v>
       </c>
@@ -5922,7 +5922,7 @@
       </c>
       <c r="F5" s="120" t="inlineStr"/>
     </row>
-    <row r="6" ht="126" customHeight="1">
+    <row r="6" ht="140" customHeight="1">
       <c r="A6" s="121" t="n">
         <v>33</v>
       </c>
@@ -5957,7 +5957,7 @@
       </c>
       <c r="F6" s="105" t="inlineStr"/>
     </row>
-    <row r="7" ht="126" customHeight="1">
+    <row r="7" ht="140" customHeight="1">
       <c r="A7" s="116" t="n">
         <v>34</v>
       </c>
@@ -6027,7 +6027,7 @@
       </c>
       <c r="F8" s="105" t="inlineStr"/>
     </row>
-    <row r="9" ht="112" customHeight="1">
+    <row r="9" ht="140" customHeight="1">
       <c r="A9" s="116" t="n">
         <v>36</v>
       </c>
@@ -6061,7 +6061,7 @@
       </c>
       <c r="F9" s="120" t="inlineStr"/>
     </row>
-    <row r="10" ht="126" customHeight="1">
+    <row r="10" ht="140" customHeight="1">
       <c r="A10" s="121" t="n">
         <v>37</v>
       </c>
@@ -6096,7 +6096,7 @@
       </c>
       <c r="F10" s="105" t="inlineStr"/>
     </row>
-    <row r="11" ht="140" customHeight="1">
+    <row r="11" ht="154" customHeight="1">
       <c r="A11" s="116" t="n">
         <v>38</v>
       </c>
@@ -6301,7 +6301,7 @@
       </c>
       <c r="F4" s="105" t="inlineStr"/>
     </row>
-    <row r="5" ht="112" customHeight="1">
+    <row r="5" ht="126" customHeight="1">
       <c r="A5" s="124" t="n">
         <v>42</v>
       </c>
@@ -6335,7 +6335,7 @@
       </c>
       <c r="F5" s="128" t="inlineStr"/>
     </row>
-    <row r="6" ht="126" customHeight="1">
+    <row r="6" ht="154" customHeight="1">
       <c r="A6" s="129" t="n">
         <v>43</v>
       </c>
@@ -6370,7 +6370,7 @@
       </c>
       <c r="F6" s="105" t="inlineStr"/>
     </row>
-    <row r="7" ht="140" customHeight="1">
+    <row r="7" ht="154" customHeight="1">
       <c r="A7" s="124" t="n">
         <v>44</v>
       </c>
@@ -6406,7 +6406,7 @@
       </c>
       <c r="F7" s="128" t="inlineStr"/>
     </row>
-    <row r="8" ht="126" customHeight="1">
+    <row r="8" ht="140" customHeight="1">
       <c r="A8" s="129" t="n">
         <v>45</v>
       </c>
@@ -6475,7 +6475,7 @@
       </c>
       <c r="F9" s="128" t="inlineStr"/>
     </row>
-    <row r="10" ht="112" customHeight="1">
+    <row r="10" ht="140" customHeight="1">
       <c r="A10" s="129" t="n">
         <v>47</v>
       </c>
@@ -6509,7 +6509,7 @@
       </c>
       <c r="F10" s="105" t="inlineStr"/>
     </row>
-    <row r="11" ht="98" customHeight="1">
+    <row r="11" ht="112" customHeight="1">
       <c r="A11" s="124" t="n">
         <v>48</v>
       </c>
@@ -6542,7 +6542,7 @@
       </c>
       <c r="F11" s="128" t="inlineStr"/>
     </row>
-    <row r="12" ht="126" customHeight="1">
+    <row r="12" ht="140" customHeight="1">
       <c r="A12" s="129" t="n">
         <v>49</v>
       </c>
@@ -6641,7 +6641,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="126" customHeight="1">
+    <row r="3" ht="140" customHeight="1">
       <c r="A3" s="132" t="n">
         <v>50</v>
       </c>
@@ -6711,7 +6711,7 @@
       </c>
       <c r="F4" s="105" t="inlineStr"/>
     </row>
-    <row r="5" ht="126" customHeight="1">
+    <row r="5" ht="168" customHeight="1">
       <c r="A5" s="132" t="n">
         <v>52</v>
       </c>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="F5" s="136" t="inlineStr"/>
     </row>
-    <row r="6" ht="84" customHeight="1">
+    <row r="6" ht="112" customHeight="1">
       <c r="A6" s="137" t="n">
         <v>53</v>
       </c>
@@ -6812,7 +6812,7 @@
       </c>
       <c r="F7" s="136" t="inlineStr"/>
     </row>
-    <row r="8" ht="112" customHeight="1">
+    <row r="8" ht="126" customHeight="1">
       <c r="A8" s="137" t="n">
         <v>55</v>
       </c>
@@ -6846,7 +6846,7 @@
       </c>
       <c r="F8" s="105" t="inlineStr"/>
     </row>
-    <row r="9" ht="98" customHeight="1">
+    <row r="9" ht="140" customHeight="1">
       <c r="A9" s="132" t="n">
         <v>56</v>
       </c>
@@ -6943,7 +6943,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="196" customHeight="1">
+    <row r="3" ht="280" customHeight="1">
       <c r="A3" s="140" t="n">
         <v>57</v>
       </c>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="F3" s="144" t="inlineStr"/>
     </row>
-    <row r="4" ht="154" customHeight="1">
+    <row r="4" ht="238" customHeight="1">
       <c r="A4" s="145" t="n">
         <v>58</v>
       </c>
@@ -7084,7 +7084,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="126" customHeight="1">
+    <row r="3" ht="168" customHeight="1">
       <c r="A3" s="148" t="n">
         <v>59</v>
       </c>
@@ -7119,7 +7119,7 @@
       </c>
       <c r="F3" s="152" t="inlineStr"/>
     </row>
-    <row r="4" ht="126" customHeight="1">
+    <row r="4" ht="210" customHeight="1">
       <c r="A4" s="153" t="n">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
feat(calendario): verifica accettazione invito e presenza evento nel calendario del destinatario
test_calendario_03.py ora accetta l'invito lato destinatario (bottone RSVP "Si"),
verifica che l'evento corretto compaia nel suo calendario (organizzatore tra i
partecipanti) e che l'organizzatore riceva la mail "Accettato: ...", tenendo
entrambe le pagine browser aperte per tutta la verifica incrociata. Aggiornati
README e testbook Excel di conseguenza.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/suite_test_pec.xlsx
+++ b/suite_test_pec.xlsx
@@ -3176,7 +3176,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="336" customHeight="1">
+    <row r="34" ht="409" customHeight="1">
       <c r="A34" s="45" t="n">
         <v>32</v>
       </c>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="E34" s="48" t="inlineStr">
         <is>
-          <t>Verifica la creazione di un evento con invito al partecipante principale e secondario, il ricevimento dell'invito lato organizzatore e la ricezione effettiva lato destinatario secondario (secondo account, seconda pagina browser).</t>
+          <t>Verifica la creazione di un evento con invito al partecipante principale e secondario, il ricevimento dell'invito lato organizzatore, la ricezione effettiva lato destinatario secondario (secondo account, seconda pagina browser), l'accettazione dell'invito da parte del destinatario, la presenza dell'evento corretto nel calendario del destinatario e la conseguente notifica di accettazione ricevuta dall'organizzatore. Le due pagine browser restano aperte contemporaneamente per tutta la verifica incrociata.</t>
         </is>
       </c>
       <c r="F34" s="49" t="inlineStr">
@@ -3210,15 +3210,19 @@
 6. Verificare il toast di conferma salvataggio evento (assert su testo IT/FR).
 7. Salvare e inviare l'invito.
 8. Navigare in In arrivo messaggi (account organizzatore) e verificare la ricevuta (assert).
-9. Aprire una seconda pagina/contesto browser, accedere con le credenziali del destinatario secondario.
+9. Aprire una seconda pagina/contesto browser (senza chiudere la prima), accedere con le credenziali del destinatario secondario.
 10. Navigare in In arrivo del destinatario secondario e attendere (polling) l'arrivo dell'email di invito.
 11. Verificare che l'invito sia effettivamente arrivato nella inbox del destinatario secondario (assert).
-12. Eliminare l'evento (cleanup lato organizzatore).</t>
+12. Aprire l'email di invito e cliccare 'Sì' per accettare la partecipazione.
+13. Navigare nel Calendario del destinatario secondario (vista Eventi), aprire l'evento con lo stesso titolo e verificare che l'organizzatore sia presente tra i partecipanti (assert), confermando che sia l'evento corretto e non un titolo omonimo.
+14. Con entrambe le pagine ancora aperte, tornare sulla pagina dell'organizzatore e attendere (polling) l'email di notifica 'Accettato: ...'.
+15. Verificare che la mail di accettazione sia arrivata nella inbox dell'organizzatore (assert).
+16. Chiudere la seconda pagina/contesto ed eliminare l'evento (cleanup lato organizzatore).</t>
         </is>
       </c>
       <c r="G34" s="50" t="inlineStr">
         <is>
-          <t>L'evento è creato con entrambi i partecipanti invitati. L'invito viene inviato come messaggio PEC ed è visibile sia nella ricevuta dell'organizzatore sia, effettivamente, nella inbox del destinatario secondario tramite un secondo account/pagina browser.</t>
+          <t>L'evento è creato con entrambi i partecipanti invitati. L'invito viene inviato come messaggio PEC ed è visibile sia nella ricevuta dell'organizzatore sia nella inbox del destinatario secondario. Dopo l'accettazione, l'evento corretto compare nel calendario del destinatario (con l'organizzatore tra i partecipanti) e l'organizzatore riceve una mail di notifica 'Accettato: ...' prima che l'evento venga eliminato.</t>
         </is>
       </c>
     </row>
@@ -5897,7 +5901,7 @@
       </c>
       <c r="F4" s="105" t="inlineStr"/>
     </row>
-    <row r="5" ht="266" customHeight="1">
+    <row r="5" ht="409" customHeight="1">
       <c r="A5" s="116" t="n">
         <v>32</v>
       </c>
@@ -5909,7 +5913,7 @@
       </c>
       <c r="C5" s="118" t="inlineStr">
         <is>
-          <t>Verifica la creazione di un evento con invito al partecipante principale e secondario, il ricevimento dell'invito lato organizzatore e la ricezione effettiva lato destinatario secondario (secondo account, seconda pagina browser).</t>
+          <t>Verifica la creazione di un evento con invito al partecipante principale e secondario, il ricevimento dell'invito lato organizzatore, la ricezione effettiva lato destinatario secondario (secondo account, seconda pagina browser), l'accettazione dell'invito da parte del destinatario, la presenza dell'evento corretto nel calendario del destinatario e la conseguente notifica di accettazione ricevuta dall'organizzatore. Le due pagine browser restano aperte contemporaneamente per tutta la verifica incrociata.</t>
         </is>
       </c>
       <c r="D5" s="119" t="inlineStr">
@@ -5922,15 +5926,19 @@
 6. Verificare il toast di conferma salvataggio evento (assert su testo IT/FR).
 7. Salvare e inviare l'invito.
 8. Navigare in In arrivo messaggi (account organizzatore) e verificare la ricevuta (assert).
-9. Aprire una seconda pagina/contesto browser, accedere con le credenziali del destinatario secondario.
+9. Aprire una seconda pagina/contesto browser (senza chiudere la prima), accedere con le credenziali del destinatario secondario.
 10. Navigare in In arrivo del destinatario secondario e attendere (polling) l'arrivo dell'email di invito.
 11. Verificare che l'invito sia effettivamente arrivato nella inbox del destinatario secondario (assert).
-12. Eliminare l'evento (cleanup lato organizzatore).</t>
+12. Aprire l'email di invito e cliccare 'Sì' per accettare la partecipazione.
+13. Navigare nel Calendario del destinatario secondario (vista Eventi), aprire l'evento con lo stesso titolo e verificare che l'organizzatore sia presente tra i partecipanti (assert), confermando che sia l'evento corretto e non un titolo omonimo.
+14. Con entrambe le pagine ancora aperte, tornare sulla pagina dell'organizzatore e attendere (polling) l'email di notifica 'Accettato: ...'.
+15. Verificare che la mail di accettazione sia arrivata nella inbox dell'organizzatore (assert).
+16. Chiudere la seconda pagina/contesto ed eliminare l'evento (cleanup lato organizzatore).</t>
         </is>
       </c>
       <c r="E5" s="50" t="inlineStr">
         <is>
-          <t>L'evento è creato con entrambi i partecipanti invitati. L'invito viene inviato come messaggio PEC ed è visibile sia nella ricevuta dell'organizzatore sia, effettivamente, nella inbox del destinatario secondario tramite un secondo account/pagina browser.</t>
+          <t>L'evento è creato con entrambi i partecipanti invitati. L'invito viene inviato come messaggio PEC ed è visibile sia nella ricevuta dell'organizzatore sia nella inbox del destinatario secondario. Dopo l'accettazione, l'evento corretto compare nel calendario del destinatario (con l'organizzatore tra i partecipanti) e l'organizzatore riceve una mail di notifica 'Accettato: ...' prima che l'evento venga eliminato.</t>
         </is>
       </c>
       <c r="F5" s="120" t="inlineStr"/>

</xml_diff>